<commit_message>
feat(export): thick separator line between guards in constraints Excel
Each guard occupies three stacked rows (בוקר/ערב/לילה) in the constraints
report, making it hard to see where one guard ends and the next begins. Add a
heavy bottom border under each guard's three-row block.

For non-merged cells the separator is drawn by _draw_guard_separator. For the
vertically-merged columns (name/phone/notes and the merged "לא זמין"/"זמין" day
cells) the thick side must be set on the merge's anchor (top-left) cell — via a
new thick_bottom param on _merge_vertical — because openpyxl derives a merged
range's outer borders from the anchor and silently overwrites a border set
directly on the bottom MergedCell.

Also regenerate the shipped sample workbook with the new look and add
scripts/generate_constraints_example.py so it can be rebuilt from the demo data.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/דוגמה_אילוצים_מאבטחים.xlsx
+++ b/דוגמה_אילוצים_מאבטחים.xlsx
@@ -88,7 +88,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -102,11 +102,17 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thick"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -117,7 +123,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -126,10 +132,10 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -140,13 +146,22 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -678,21 +693,21 @@
       <c r="K6" s="9" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="n"/>
-      <c r="B7" s="9" t="n"/>
-      <c r="C7" s="13" t="inlineStr">
+      <c r="A7" s="13" t="n"/>
+      <c r="B7" s="13" t="n"/>
+      <c r="C7" s="14" t="inlineStr">
         <is>
           <t>לילה</t>
         </is>
       </c>
-      <c r="D7" s="11" t="n"/>
-      <c r="E7" s="11" t="n"/>
-      <c r="F7" s="11" t="n"/>
-      <c r="G7" s="11" t="n"/>
-      <c r="H7" s="11" t="n"/>
-      <c r="I7" s="12" t="n"/>
-      <c r="J7" s="12" t="n"/>
-      <c r="K7" s="9" t="n"/>
+      <c r="D7" s="15" t="n"/>
+      <c r="E7" s="15" t="n"/>
+      <c r="F7" s="15" t="n"/>
+      <c r="G7" s="15" t="n"/>
+      <c r="H7" s="15" t="n"/>
+      <c r="I7" s="16" t="n"/>
+      <c r="J7" s="16" t="n"/>
+      <c r="K7" s="13" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -753,41 +768,41 @@
       <c r="K9" s="9" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="9" t="n"/>
-      <c r="B10" s="9" t="n"/>
-      <c r="C10" s="13" t="inlineStr">
+      <c r="A10" s="13" t="n"/>
+      <c r="B10" s="13" t="n"/>
+      <c r="C10" s="14" t="inlineStr">
         <is>
           <t>לילה</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="D10" s="17" t="inlineStr">
         <is>
           <t>23:00–07:00</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="E10" s="17" t="inlineStr">
         <is>
           <t>23:00–07:00</t>
         </is>
       </c>
-      <c r="F10" s="12" t="n"/>
-      <c r="G10" s="11" t="n"/>
-      <c r="H10" s="6" t="inlineStr">
+      <c r="F10" s="16" t="n"/>
+      <c r="G10" s="15" t="n"/>
+      <c r="H10" s="17" t="inlineStr">
         <is>
           <t>23:00–07:00</t>
         </is>
       </c>
-      <c r="I10" s="6" t="inlineStr">
+      <c r="I10" s="17" t="inlineStr">
         <is>
           <t>23:00–07:00</t>
         </is>
       </c>
-      <c r="J10" s="6" t="inlineStr">
+      <c r="J10" s="17" t="inlineStr">
         <is>
           <t>23:00–07:00</t>
         </is>
       </c>
-      <c r="K10" s="9" t="n"/>
+      <c r="K10" s="13" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -868,21 +883,21 @@
       <c r="K12" s="9" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="9" t="n"/>
-      <c r="B13" s="9" t="n"/>
-      <c r="C13" s="13" t="inlineStr">
+      <c r="A13" s="13" t="n"/>
+      <c r="B13" s="13" t="n"/>
+      <c r="C13" s="14" t="inlineStr">
         <is>
           <t>לילה</t>
         </is>
       </c>
-      <c r="D13" s="12" t="n"/>
-      <c r="E13" s="12" t="n"/>
-      <c r="F13" s="11" t="n"/>
-      <c r="G13" s="11" t="n"/>
-      <c r="H13" s="11" t="n"/>
-      <c r="I13" s="11" t="n"/>
-      <c r="J13" s="12" t="n"/>
-      <c r="K13" s="9" t="n"/>
+      <c r="D13" s="16" t="n"/>
+      <c r="E13" s="16" t="n"/>
+      <c r="F13" s="15" t="n"/>
+      <c r="G13" s="15" t="n"/>
+      <c r="H13" s="15" t="n"/>
+      <c r="I13" s="15" t="n"/>
+      <c r="J13" s="16" t="n"/>
+      <c r="K13" s="13" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -922,7 +937,7 @@
           <t>07:00–14:00</t>
         </is>
       </c>
-      <c r="J14" s="14" t="inlineStr">
+      <c r="J14" s="18" t="inlineStr">
         <is>
           <t>זמין</t>
         </is>
@@ -959,29 +974,29 @@
         </is>
       </c>
       <c r="I15" s="11" t="n"/>
-      <c r="J15" s="15" t="n"/>
+      <c r="J15" s="19" t="n"/>
       <c r="K15" s="9" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="9" t="n"/>
-      <c r="B16" s="9" t="n"/>
-      <c r="C16" s="13" t="inlineStr">
+      <c r="A16" s="13" t="n"/>
+      <c r="B16" s="13" t="n"/>
+      <c r="C16" s="14" t="inlineStr">
         <is>
           <t>לילה</t>
         </is>
       </c>
-      <c r="D16" s="11" t="n"/>
-      <c r="E16" s="11" t="n"/>
-      <c r="F16" s="11" t="n"/>
-      <c r="G16" s="6" t="inlineStr">
+      <c r="D16" s="15" t="n"/>
+      <c r="E16" s="15" t="n"/>
+      <c r="F16" s="15" t="n"/>
+      <c r="G16" s="17" t="inlineStr">
         <is>
           <t>23:00–07:00</t>
         </is>
       </c>
-      <c r="H16" s="11" t="n"/>
-      <c r="I16" s="11" t="n"/>
-      <c r="J16" s="15" t="n"/>
-      <c r="K16" s="9" t="n"/>
+      <c r="H16" s="15" t="n"/>
+      <c r="I16" s="15" t="n"/>
+      <c r="J16" s="20" t="n"/>
+      <c r="K16" s="13" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -1054,21 +1069,21 @@
       <c r="K18" s="9" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="9" t="n"/>
-      <c r="B19" s="9" t="n"/>
-      <c r="C19" s="13" t="inlineStr">
+      <c r="A19" s="13" t="n"/>
+      <c r="B19" s="13" t="n"/>
+      <c r="C19" s="14" t="inlineStr">
         <is>
           <t>לילה</t>
         </is>
       </c>
-      <c r="D19" s="11" t="n"/>
-      <c r="E19" s="12" t="n"/>
-      <c r="F19" s="12" t="n"/>
-      <c r="G19" s="11" t="n"/>
-      <c r="H19" s="12" t="n"/>
-      <c r="I19" s="12" t="n"/>
-      <c r="J19" s="11" t="n"/>
-      <c r="K19" s="9" t="n"/>
+      <c r="D19" s="15" t="n"/>
+      <c r="E19" s="16" t="n"/>
+      <c r="F19" s="16" t="n"/>
+      <c r="G19" s="15" t="n"/>
+      <c r="H19" s="16" t="n"/>
+      <c r="I19" s="16" t="n"/>
+      <c r="J19" s="15" t="n"/>
+      <c r="K19" s="13" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="28">

</xml_diff>